<commit_message>
start on module to provide model information
</commit_message>
<xml_diff>
--- a/data-raw/project_texts.xlsx
+++ b/data-raw/project_texts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\neilm\Projects\b_useful\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F4A866A-7BA4-4424-8217-47BC6DFF66F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB493EBE-2960-4678-927A-D484D3241616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" firstSheet="1" activeTab="3" xr2:uid="{B3A1738F-4730-4C3D-B31B-830F2610B29E}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" firstSheet="6" activeTab="9" xr2:uid="{B3A1738F-4730-4C3D-B31B-830F2610B29E}"/>
   </bookViews>
   <sheets>
     <sheet name="landing_page" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,10 @@
     <sheet name="tooltips" sheetId="6" r:id="rId5"/>
     <sheet name="downloads" sheetId="9" r:id="rId6"/>
     <sheet name="sources" sheetId="7" r:id="rId7"/>
+    <sheet name="nea_model" sheetId="10" r:id="rId8"/>
+    <sheet name="iceland_model" sheetId="11" r:id="rId9"/>
+    <sheet name="wmed_model" sheetId="12" r:id="rId10"/>
+    <sheet name="emed_model" sheetId="13" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="99">
   <si>
     <t>text</t>
   </si>
@@ -335,11 +339,6 @@
 &lt;li&gt;Model Diagnostics&lt;/li&gt;</t>
   </si>
   <si>
-    <t>B-USEFUL's model outputs are available the &lt;a hfef="https://creativecommons.org/licenses/by/4.0/ "&gt; CC BY 4.0 license&lt;/a&gt;&lt;br&gt;
-Please feel free to download and use the data, providing attribution to the authors.&lt;br&gt;&lt;br&gt;
-The data is available as a zipfile bundle per model. Select from the models to see the available data and access the download link.</t>
-  </si>
-  <si>
     <t>Filtered spatial patterns
 of  {taxon} {diversity_indicator} in the {ecoregion}. Only locations that meet all user defined selection criteria are retained: &lt;br&gt;
 &lt;strong&gt;Species Richness Percentiles:&lt;/strong&gt; {rich_pct};
@@ -351,6 +350,412 @@
 &lt;strong&gt;Functional Divergence Percentiles:&lt;/strong&gt; {fdiv_pct}.
 &lt;br&gt;The indicators are
 based on model predictions for the selected year: {yr}.</t>
+  </si>
+  <si>
+    <t>sdm_occurrence</t>
+  </si>
+  <si>
+    <t>sdm_biomass</t>
+  </si>
+  <si>
+    <t>sdm_abundance</t>
+  </si>
+  <si>
+    <t>Modelled probability of occurrence {sp} for {yr} in the {case} ecoregion.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modelled biomass of {sp} for {yr} in the {case} ecoregion (Individuals / km&lt;sup&gt;2&lt;/sup&gt;). </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modelled abundance of {sp} for {yr} in the {case} ecoregion (kg / km&lt;sup&gt;2&lt;/sup&gt;). </t>
+  </si>
+  <si>
+    <t>B-USEFUL's model outputs are available the &lt;a hfef="https://creativecommons.org/licenses/by/4.0/ "&gt; CC BY 4.0 license&lt;/a&gt;&lt;br&gt;
+Please feel free to download and use the data, providing attribution to the authors.&lt;br&gt;&lt;br&gt;
+The recommended citation for use of B-USEFUL data is: &lt;br&gt;&lt;br&gt;
+B-USEFUL. Report on temporal trends and spatial patterns of multiple biodiversity indicators. Technical University of Denmark (2025). Martin Lindegren, Manuel Hidalgo, Marcel Montanyes, Federico Maioli, Benjamin Weigel,
+Daniel van Denderen, Gleb Tikhnov, Otso Ovaskainen, Baptiste Degueurce, Tim Jimenez,
+Francesco Golin, Ingibjörg G. Jónsdóttir, Haseeb Randhawa, Julian Burgos, Walter Zupa,
+Antonella Consiglio, Matteo Chiarini, Maria Teresa Spedicato, Patricia Puerta, Alicia Gran,
+Shannon Moore, Laurene Pecuchet, Murray Thompson, Lily Greig, Keith Cooper, Georg
+Engelhard, Justin Tiago, Marcel Rozemeijer, Sofia Henriques, André Martins, Corina Chaves,
+Rita Vasconcelos, Teresa Moura. &lt;br&gt;&lt;br&gt;
+The data is available as a zipfile bundle per model. Select from the models to see the available data and access the download link.</t>
+  </si>
+  <si>
+    <t>authors</t>
+  </si>
+  <si>
+    <t>Marcel Montanyès, Benjamin Weigel, Federico Maioli, Gleb Tikhonov, Pieter Daniël
+van Denderen, Otso Ovaskainen, Martin Lindegren</t>
+  </si>
+  <si>
+    <t>model</t>
+  </si>
+  <si>
+    <t>diagnostics</t>
+  </si>
+  <si>
+    <t>area_and_data</t>
+  </si>
+  <si>
+    <t>We gathered a comprehensive data set on fish species distribution and biomass from 13 scientific bottom-trawl surveys conducted across the North and North-east Atlantic Ocean (Appendix 1; Table S1). The data set encompass 90,029 unique hauls spanning 33 years (1989-2021), thus capturing the active period for most surveys and providing an extensive spatio-temporal coverage of our study area (Figure 3.1.1). We focused our analysis solely on fish taxa (i.e., Elasmobranchii, Actinopteri, Holocephali, Myxini, Petromyzonti and Teleostei) identified at the species level and that exhibited a minimum prevalence of 0.1% (i.e., &gt; 90 occurrences), resulting in a selection of 151 species. The species names were crossreferenced and updated using the World Register of Marine Species (WoRMS Editorial Board 2022). For each of the hauls we recorded the presence-absence of species, as well as their biomass standardized for sampling area (km2) and trawl gear catchability following methodologies detailed in previous studies (van Denderen et al. 2023; Maureaud et al. 2019; Walker et al. 2017).</t>
+  </si>
+  <si>
+    <t>traits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To account for functional (trait) aspects of biodiversity, we selected 6 traits that broadly represent the life history, reproduction, morphology and diet of species (Dencker et al. 2017) following a formal framework developed for other marine organisms (Litchman, Ohman, and Kiørboe 2013). Trait information was retrieved from the database by Beukhof et al. (2019). The life history of each species was characterized by two parameters: age of maturity (in years) and the von Bertalanffy growth coefficient K (measured in year-1), while the reproductive traits were represented by offspring size, i.e. egg diameter (measured in mm). Morphological characteristics were assessed through maximum length (in cm) and the caudal fin aspect ratio as a proxy for mobility. Lastly, we considered diet by including the
+trophic level of each species. </t>
+  </si>
+  <si>
+    <t>environment</t>
+  </si>
+  <si>
+    <t>To represent the environmental conditions at each unique haul, we retrieved environmental and physical variables from the model re-analysis products of the NEMO-MEDUSA model (Gurvan et al. 2022; Yool et al. 2013). This provided us with surface and bottom details concerning temperature (ºC), salinity (PSU), detritus concentration (mmol N per m3), chlorophyll a concentration (Chl a; mmol N per m3) and dissolved inorganic nitrogen concentration (DIN; mmol N per m3), as well as depth (m). Additionally, we computed the annual standard deviation for temperature, salinity, and Chl
+a at each location, as a proxy for seasonal variation (Beukhof et al. 2019; Dencker et al. 2017; Maureaud et al. 2019). Due to the lack of available long-term data on fishing effort throughout the area, the potential effects of commercial fishing were not explicitly accounted for. However, previous large-scale studies on marine fish communities in the area found no, or only weak effects on the species distribution and community trait composition (Beukhof et al. 2019; Dencker et al. 2017). After checking for potential collinearity we omitted highly correlated variables, i.e., with Pearson coefficient &gt; 0.7 (Appendix 1; Figure S1). The final set of environmental covariates comprises sea bottom temperature (SBT), SBT seasonality, sea bottom salinity (SBS), SBS seasonality, seafloor detritus, surface DIN, surface Chl a, surface Chl a seasonality, seafloor Chl a seasonality, and depth.</t>
+  </si>
+  <si>
+    <t>We employed HMSC to model the fish communities, treating each unique sample event as a response variable. Given the zero-inflated nature of the data, we adopted a hurdle approach. This involved utilizing one model for presence-absence (probit regression) and another model for biomass conditional on presence (log-linear regression). As fixed effects we incorporated the environmental covariates detailed above, including quadratic terms for sea bottom temperature (SBT) and sea bottom salinity (SBS) to account for potential nonlinear species' responses. To account for potential seasonal differences in distribution and biomass (i.e., linked to migrations and spawning) we further included spring/summer and autumn/winter as a fixed factor. In addition to the fixed effects, the models encompassed spatially- (Ovaskainen et al. 2016) and temporally (yearly) structured latent variables. Spatial units were represented by hexagonal cells (N=574 cells), each covering an area of 7,774 km2. To determine the relative importance of the environmental covariates we partitioned the explained variation among the fixed and random effects (Ovaskainen et al. 2017; Ovaskainen and Abrego 2020). The model was fitted with four Markov chain Monte Carlo (MCMC) chains taking 250 samples per chain, resulting in 1,000 posterior samples. The thinning applied was specific to each model with the aim of achieving a good model convergence with a reasonable use of computational resources. We assessed MCMC convergence by examining the potential scale reduction factors (PSRFs; Gelman and Rubin 1992) of model parameters where values &lt;1.1 indicate satisfactory convergence (Tikhonov et al. 2020). To assess the predictive performance of our models we partitioned the data into three decades (1989- 1999, 2000-2009, 2010-2021) and trained separate models on each decade. To evaluate the explanatory power of these trained models, we employed metrics such as AUC and Tjur R2 for species presence-absence, R2 for biomass conditional on presence, and root mean square error (RMSE) for both (Ovaskainen &amp; Abrego, 2020). Subsequently, we tested the models on the remaining decades to assess their out-of-sample predictive performances.</t>
+  </si>
+  <si>
+    <t>Francesco Golin, Haseeb Randhawa, Federico Maioli, Martin Lindegren, Julian
+Burgos, Ingibjörg G. Jónsdóttir</t>
+  </si>
+  <si>
+    <t>The data for this study has been collected through bottom trawling as part of the Icelandic
+Groundfish Survey (SMB) and the Autumn Groundfish Survey (SMH), both of which are carried
+out by the Marine and Freshwater Research Institute of Iceland (Figure 3.5.1). The temporal
+span of the data is 1996 – 2024, while the sampling points span between 62° 12' 50.4" N and
+68° 19' 43.2" N in latitude, 31° 32' 12.6" W and 9° 36' 49.8" W in longitude, and 30-1500 m in
+depth. For this study, only data concerning species belonging to the classes Actinopterygii,
+Elasmobranchii, Holocephali, Myxinii and Petromyzontii have been considered. The data went
+through a quality check procedure during which invalid hauls and invalid species records have
+been removed. Additionally, rare species with less than 10 occurrence records over space
+(ICES rectangles), time (years), and with less than 1% occurrence in the dataset have been
+removed (140 species). Pelagic and bathypelagic species (19 in total) were also removed from
+the analysis, as their lower catchability in bottom trawled gear can lead to the
+underestimation of their abundance (Walker et al. 2017). The benthopelagic species Clupea
+harengus, Cyclopterus lumpus and Mallotus villosus were also removed due to possible large
+geographical variability in abundance given by their mobility. Therefore, the analysis included
+82 species found in 25 911 samples (Figure 3.5.1). Species abundance was expressed as kg/km2. These estimates of density were calculated using
+information on the species-specific number of individuals and length distribution found in
+each sample and the species-specific coefficients of the length-weight relationship available
+from FishBase (Froese and Pauly 2024). These estimates were then adjusted using coefficients
+of fishing gear efficiency provided in the Supplementary Information of Walker et al. (2017).</t>
+  </si>
+  <si>
+    <t>To characterize species in terms of their morphology, life history, reproduction and diet
+(Dencker et al. 2017) we selected 7 ecological traits to be included in the models. Morphology
+was described by maximum length (m) and the aspect ratio of the caudal fin, which
+constituted a proxy for mobility. Life history was described by the age of maturity (years) and
+by the von Bertalanffy growth coefficient (K) (year-1). Life history was described by the age of
+maturity and by fecundity (number of offspring), while dietary aspects were described by the
+trophic level. Finally, the position usually occupied in the water column was included as a
+categorical variable with three levels: demersal, bathydemersal and benthopelagic. Trait
+information was gathered for each species using available datasets (Beukhof et al. 2019,
+Thorson et al. 2017) and supplemented with information found in recent literature
+(Emblemsvåg et al. 2020). If no information could be found for a specific trait, the Genus or
+Family average was used. Furthermore, to estimate the influence of taxonomically structured
+traits on species niches, taxonomic information was retrieved from WoRMS (Ahyong et al.
+2025) and included in the model.</t>
+  </si>
+  <si>
+    <t>Information on the physical and biogeochemical environment were sourced from data
+products by Copernicus Marine (Copernicus Marine Service 2025a and 2025b). These provided
+monthly averages of sea bottom temperature (SBT) (°C), sea bottom salinity (/103), chlorophyll
+a concentration (at surface, mg/m3), dissolved oxygen (mmol/m3), nitrate concentration (at
+surface, mmol/m3), phosphate concentration (at surface, mmol/m3), silicate concentration (at
+surface, mmol/m3) and net primary production of biomass (at surface, expressed as mg carbon
+/m3/day). The annual standard deviation of sea bottom temperature (SD SBT) (°C) was
+included as a measure of seasonality and stability of the environmental conditions at each
+sampling location. Information on the site of sampling included depth (m), mean sea bottom
+slope for a 5km radius around the sampling site (°), and the mean fishing effort by bottom
+trawling for the year past the month of sampling and a 20 km radius. This was expressed as a
+ratio between the swept are and the area of a cell, following a methodology akin to the one
+found in Gerritsen et al. 2013. Data on sea bottom slope was calculated using bathymetric
+information by the R package marmap (Pante et al. 2023) and the package terra (Hijmans
+2025), while data on fishing effort was retrieved from logbook data property of the Icelandic
+Ministry of Fishery (Fiskistofa 2025). To capture possible variability in occurrence and
+abundance due to diel migration, time of sampling (expressed as hours from solar noon) was
+included in the models. The above-mentioned environmental covariates were tested for
+multicollinearity, and when two variables had a correlation &gt;0.7 or &lt;-0.7, only the one least
+correlated with the other variables was kept for analysis (Figure S1). The only exception was
+nitrate concentration, which was excluded to avoid overfitting, since chlorophyll
+concentration was deemed sufficient to constitute a proxy of primary productivity. Therefore,
+the set of variables with limited reciprocal correlation were SBT, SD SBT, salinity, chlorophyll
+concentration, oxygen concentration, depth, mean slope, fishing effort, and time from solar
+noon.</t>
+  </si>
+  <si>
+    <t>To model the response of the selected species to the environment, the hierarchical modelling
+of species community (HMSC) framework was used (Ovaskainen et al. 2017). Due to the zero
+inflated nature of the data, a hurdle approach was used. This involves producing a presenceabsence
+model, denominated here as PA model, and an abundance conditional on presence
+model, the ABU model. The models were fitted using the default priors reported in the
+Supporting Information of Tikhonov et al. (2020). Four Markov chain Monte Carlo (MCMC)
+chains were run using the high-performance computing implementation described in Rahman
+et al. (2024). Each chain collected 250 samples, resulting in a total of 1000 posterior samples.
+We applied applied a thinning of 250, resulting in 93 750 iterations per chain, of which the
+first 31 250 were discarded as burn-in. MCMC convergence was evaluated using the potential
+scale reduction factor (PSRF) (Gelman and Rubin 1992), and it was considered satisfactory
+when it did not exceed 1.1 (Tikhonov et al. 2020). Three species (Centroscyllium fabricii,
+Deania calceus, Notacanthus chemnitzii) were removed at this step due to poor chain
+convergence for many of their parametres, which affected the overall performance of the
+models. As fixed effects we included SBT, SD SBT, salinity, chlorophyll concentration, depth,
+mean slope, fishing effort and time from solar noon. Oxygen concentration was ultimately
+excluded as its parameter estimates suffered from poor convergence. Anyway, it was deemed
+unlikely that oxygen concentration would have influenced the distribution of the chosen
+species, as no site had an estimated oxygen concentration close to hypoxic conditions
+(commonly defined as concentrations lower than 63 mmol/m3) (Rabalais et al., 2002), with
+the range of available measurements being included between 201 mmol/m3 and 358
+mmol/m3. Furthermore, to accommodate non-linear responses in species niches to SBT and
+depth, quadratic terms were included for both of these variables. Finally, mean slope was logtransformed
+to stabilize variance and ensure model convergence. In addition to the fixed
+effects, the models included a spatial and a temporal random effect. The unit of the spatial
+random effect was constituted by hexagonal grid cells (n = 30) with a distance of 200km
+between their centres (see Figure 3.5.1). The year of sample collection constituted the unit of
+the temporal random effect. The random effects were treated independently from each
+other. The number of latent variables to be produced by the model was limited to a minimum
+of 1 and a maximum of 5. Latent variables are used in the HMSC framework to estimate the
+parameters of residual association between pairs of species (Ovaskainen and Abrego 2020).
+Model performance was evaluated both as explanatory and predictive power through a 5-fold
+cross-validation. The under the receiver operating characteristic curve (AUC), Tjur’s R2 and the
+root mean square error (RMSE) were used to evaluate the performance of the PA model, while
+R2 and RMSE were used to evaluate the performance of the ABU model.</t>
+  </si>
+  <si>
+    <t>Walter Zupa, Antonella Consiglio, Matteo Chiarini, Maria Teresa Spedicato</t>
+  </si>
+  <si>
+    <t>Data on the occurrence and abundance of demersal species were obtained from the
+Mediterranean International Bottom Trawl Survey MEDITS (Bertrand et al., 2002; Spedicato
+et al., 2019) conducted annually from May to July since 1994, recently under the EU Data
+Collection Framework (DCF; EU, (EU) 2017/1004). The survey applies a stratified random
+sampling scheme, with haul allocation proportional to the surface area of 5 depth strata
+(covering the bathymetrical range from 10m to 800m). The analyses focused on nine
+Geographical Sub-Areas (GSAs; GFCM, 2009) of the Central and Eastern Mediterranean Sea,
+specifically: GSA 15 (Malta), GSA 16 (Southern Sicily), GSA 17 (Northern Adriatic Sea), GSA 18
+(Southern Adriatic Sea), GSA 19 (Western Ionian Sea), GSA 20 (Eastern Ionian Sea), GSA 22
+(Aegean Sea), GSA 23 (Crete), and GSA 25 (Cyprus), as illustrated in Figure 3.6.1. The selected
+spatial domain covers approximately 378,852 km2 with, on average, about 577 sampling
+stations per year. The selected temporal range for the analysis spans from 1999 to 2021 to
+provide comprehensive coverage of environmental drivers used in modeling. Although the
+MEDITS survey has been conducted regularly on an annual basis, some gaps in temporal
+continuity occurred in some GSAs, such as GSA 15 and GSA 25, where sampling began in 2005,
+and some annual gaps between 2009 and 2013 in GSAs 20, 22, and 23. The survey is conducted
+in each GSA using the GOC 73 trawl gear, which is equipped with a 20 mm stretched mesh
+codend (Bertrand et al., 2002; Spedicato et al., 2019), allowing for the capture of small-sized
+individuals. Once onboard, all specimens exceeding 1 cm in size are taxonomically identified,
+and both their number and total biomass are recorded. This procedure generates a consistent
+dataset that supports the calculation of standardized abundance indices (expressed as N/km²)
+across hauls. &lt;br&gt;To ensure the quality of data used for the analysis, a multiple and comprehensive data
+validation procedure was applied on MEDITS data using the R package RoME
+(https://github.com/COISPA/RoME), routinely adopted by the MEDITS coordination group
+and embedded in the newly developed Med&amp;BS RDBFIS regional database in the
+Mediterranean (https://medbsrdb.eu/), extensively checked by experts in the QualiTrain EU
+project (EASME/EMFF/2020/OP/021). This process allows the users to easily identify the
+presence of inconsistencies in the source data, such as haul position, taxonomic classification,
+measure units, number of individuals caught, and their relative weights, which could likely
+affect the results of the modeling analysis. Consequently, data correction procedures were
+carried out, particularly oriented to address issues linked to the estimation of the sampling
+positions and of the abundance indices at the species level. To define the species pool used in
+the HMSC modeling, we calculated the occurrence and frequency of all taxa recorded in the
+catches of the dataset across all hauls of the geographical domain of the study. Species
+belonging to fish (A), decapod crustaceans (B), and cephalopods (C) were retained. The initial
+MEDITS dataset covering the study area comprised a total of 599 taxa, including 371 fish
+species (of which 321 were teleosts and 50 elasmobranchs) alongside 47 cephalopod species
+and 181 crustacean taxa. For the main analysis, we selected species with frequency of
+occurrence &gt; 1%, resulting in a final list of 184 taxa. A subsequent screening based on the
+availability of trait information led to a further reduction of the dataset, retaining 158 taxa for
+modeling purposes (120 fish, 18 crustaceans, and 20 cephalopods).</t>
+  </si>
+  <si>
+    <t>In parallel with the species occurrence and abundance, a comprehensive life-history trait
+database was developed ad hoc, as reported in the Deliverable D2.2 (https://buseful.
+eu/library/deliverables/; Spedicato et al., 2024), including 15 different traits (9
+continuous and 6 categorical). Trait databases for crustaceans and cephalopods were
+compiled, drawing primarily from SeaLifeBase (Palomares &amp; Pauly, 2022), while for fish, the
+trait dataset was assembled mostly based on Beukhof et al. (2019) complemented by FishBase
+(Froese, 2005), and through phylogenetic imputation using the R package phylosem (Thorson
+&amp; van der Bijl, 2023). The traits database was finally composed of references for 363 fish taxa,
+72 crustaceans, and 62 cephalopods.</t>
+  </si>
+  <si>
+    <t>To characterize the environmental conditions at each
+sampling location, we extracted a comprehensive set of physical and biogeochemical variables
+from the Copernicus Marine Environment Monitoring Service (CMEMS)
+(https://marine.copernicus.eu) using the reanalysis products with a monthly temporal
+resolution and a spatial resolution of 1/24° (~0.042°). Specifically, we used the product
+MEDSEA_MULTIYEAR_PHY_006_004 (Escudier et al., 2021) to retrieve sea surface and bottom
+temperature (°C) and salinity (PSU), and the product MEDSEA_MULTIYEAR_BGC_006_008
+(Cossarini et al., 2021) for surface chlorophyll-a concentration (mg m⁻³), net primary
+production (mmol N m⁻³ day⁻¹), nitrate (mmol N m⁻³), phosphate (mmol P m⁻³), dissolved
+oxygen (mmol O₂ m⁻³), and phytoplankton concentration (mmol N m⁻³). In addition, current
+velocity data were used to derive eastward and northward components of horizontal
+circulation. Furthermore, seabed substrate classification was retrieved from EMODnet
+Geology (European Marine Observation and Data network; www.emodnet-geology.eu), using
+the EUSeaMap 2023 Broad-Scale Predictive Habitat Map for Europe product (Vasquez et al.,
+2023), whereas bathymetry product tiles (EMODnet Bathymetry portal,
+http://www.emodnet-bathymetry.eu) were used to retrieve depth information. In addition,
+other pressure drivers were explored in the models’ setup, such as the gravity index (Cinner
+et al., 2018), the fishing pressure index (FPI) estimated with the application of multi-criteria decision analysis (MCDA) (Kavadas et al., 2015) and the fishing effort information provided by
+DCF Fisheries Dependent Information (FDI), spatially disaggregated by means of a fishing
+footprint derived from Global Fishing Watch (GFW). Before the model fitting, collinearity
+among environmental covariates was assessed using Pearson’s correlation matrix (Annex 6,
+Figure S1). Only predictors with pairwise correlation coefficients below 0.7 were retained as a
+conservative rule of thumb (Dormann et al., 2013), to minimize redundancy and avoid strong
+collinearity.</t>
+  </si>
+  <si>
+    <t>The HMSC framework was employed to model and investigate the drivers and community
+responses acting on the Mediterranean demersal communities through the R package Hmsc
+version 3.3-4 (Ovaskainen et al., 2017; Tikhonov et al., 2020). Due to the zero-inflated
+distribution of the data, a hurdle approach involving two separate models was adopted: a
+presence–absence model (occurrence) based on a probit distribution combined with an
+abundance conditional on presence model (abundance model). The abundance models were
+tested using different distributions, although the normal distribution was retained as it
+provided the best fitting performance. Two different hurdle models were finally produced:
+one using the whole time series (WTS), spanning from 1999 to 2021, and another using a
+shortened time series (2012–2021) that allowed the inclusion of fishing effort (FE) derived
+from DCF FDI data, spatially disaggregated using the GFW fishing footprint, which was not
+tested in the WTS models. Each model included both random and fixed effects. The former
+was selected to account for the spatial and temporal variations (by means of the inclusion of
+the grid cells and the year effects) not directly incorporated as fixed components. As fixed
+effects, bottom temperature, bottom salinity, depth, and chlorophyll-a concentration were
+finally retained in both WTS and FE models. To account for potential non-linear species–
+environment relationships, for both models, a second-degree polynomial function was
+applied to depth, for the occurrence sub-models, and extended to all other environmental
+covariates for the abundance models, except for chlorophyll-a. Chlorophyll-a concentration
+and fishing effort (for the FE model) were log-transformed to reduce variability and to improve
+the linearity of their relationship with the species response.&lt;br&gt;
+To account for interspecific variation in ecological strategies to environmental variables and
+reduce computational performance, a set of biologically meaningful traits was selected and
+incorporated into the models. The retained traits included maximum length, longevity, depth
+preference, temperature preference, and trophic level, and were applied consistently across
+taxonomic groups, including fishes, crustaceans, and cephalopods. These traits were selected
+based on their ecological relevance in structuring demersal communities and mediating
+responses to external pressure drivers. Maximum body length and longevity are key life history
+traits associated with species' reproductive output, population turnover, and
+sensitivity to exploitation (Hiddink et al., 2019; Quesne &amp; Jennings, 2012). Depth and
+temperature preferences reflect species’ niche and are critical traits determining the spatial
+distribution (Polo et al., 2025; Stuart-Smith et al., 2015). Trophic level situates species within
+the food web and is important for understanding predator–prey interactions (Romanuk et al.,
+2011). Four Markov Chain Monte Carlo (MCMC) chains were run, each drawing 250 posterior
+samples, for a total of 1000 samples. Thinning intervals were thus adjusted for each model
+individually to optimise convergence diagnostics, while ensuring computational feasibility, finally adopting a thinning interval of 2000. To ensure that the chains reached their stationary
+distribution before posterior sampling, a burn-in phase of 250,000 iterations (transients) was
+applied. As a result, each chain executed a total of 750,000 iterations (250,000 burn-in +
+500,000 sampling), yielding an overall computational effort of 3 million iterations across the
+four chains. This modeling setup adheres to widely accepted practices in Bayesian inference,
+where sufficient burn-in and thinning are essential to reduce the impact of initialisation and
+autocorrelation (Geyer, 2011; Margossian et al., 2023). Convergence of the MCMC was
+assessed by evaluating the Potential Scale Reduction Factor (PSRF; Gelman &amp; Rubin, 1992) of
+model parameters, with convergence considered satisfactory when the mean PSRF values do
+not exceed 1.1 (Tikhonov et al., 2020). Convergence of the MCMC chains was further assessed
+using the Geweke diagnostic (Geweke, 1992) for each model parameter, and convergence was
+considered satisfactory when |z| &lt; 1.96. The model performances were evaluated as both
+explanatory and predictive power through a 4-fold cross-validation. In each fold, the models
+were trained on 75% of the data and tested on the remaining 25%, iteratively covering the
+entire dataset. To quantify model performance, a set of complementary metrics was used,
+tailored to the nature of the models. For the occurrence model the following metrics were
+used: the area under the operating characteristic curve (AUC) and Tjur’s coefficient of
+discrimination (Tjur R²), a robust measure for binary response models that reflects the
+difference in predicted probabilities between observed presences and absences (Tjur, 2009).
+For the abundance (conditional-on-presence) model, the R² was used instead, while in both
+models the root mean square error (RMSE) was estimated as an indicator of the average
+deviation between observed and predicted values. All the statistical analyses were conducted
+in R software version 4.4.1 (R Core Team, 2024). The model runs and the cross-validation were
+performed on the DRAGO high-performance computing (HPC) cluster hosted by the Consejo
+Superior de Investigaciones Científicas (CSIC), exploiting the HMSC-HPC implementation using
+NVIDIA A100 40GB GPUs. For each cross-validation fold and MCMC chain, independent jobs
+were launched in parallel, allowing efficient scaling of the workload across the cluster.
+Based on the models’ predictions a set of biodiversity indicators was estimated. Taxonomic
+richness was assessed as the total number of species present at each site, considering only
+those species with an occurrence probability equal to or greater than 0.2. This threshold was
+chosen to avoid excluding rare species that typically exhibit low predicted occurrence
+probabilities, aligning with other studies that favor more inclusive thresholds (Chou et al.,
+2020; Linhoss and Mickle, 2022). The Shannon diversity index (H') was calculated using the R
+package vegan. Pielou’s evenness index (J') was computed as the ratio between the Shannon
+index and the natural logarithm of species richness. To quantify functional diversity, we
+calculated functional richness (FRic) and functional evenness (FEve) by constructing a
+multidimensional trait space. This was achieved through a Principal Coordinates Analysis
+(PCoA) based on Gower distances between species traits (Legendre and Legendre, 1998).
+These metrics describe the extent to which species occupy the available functional trait space
+within the community, and the uniformity of biomass distribution across that space (Mouillot
+et al., 2013). We retained the first three Principal Coordinates (PCs), with a cumulative
+explained variance of 83%.</t>
+  </si>
+  <si>
+    <t>Patricia Puerta, Alicia Gran, Manuel Hidalgo</t>
+  </si>
+  <si>
+    <t>We combined seabed, oceanographic and fishing pressure variables to account for spatial
+environmental and local anthropogenic impact gradients. The selection of the 6 final variables
+was based on Pearson correlations &lt;0.65 and Variance Inflation Factor values &lt;3 (VIF, Zuur et
+al. 2010) to avoid cross-correlation and collinearity, respectively. Main seabed substrate was
+obtained from the broad-scale seabed habitat map for Europe (EUSeaMap; Vasquez et al.
+2023) of the European Marine Observation Data Network (EMODnet), re-scaled to 0.042° grid
+cell, and simplified to five categories: posidonia (Posidonia oceanica meadows), hardsubstrate
+(rock or other hard-substrates), sand, mud and mixed sediment (coarse and mixed
+sediment). As oceanographic variables, monthly average of surface (SST) and bottom
+(botTemp) temperatures (°C), surface (so) and bottom (botso) salinity and chlorophyl (Chl)
+concentration (μg l−1) were obtained from the Copernicus Marine Service Data at 0.042°
+hexagonal grid cell (Nigam et al. 2021, Teruzzi et al. 2021). Finally, a fishing pressure index
+(FPI) to account for trawling, purse-seine and small-scale fisheries footprint was included
+(Kavada et al. 2015).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">We used annual data of the Mediterranean International Bottom Trawl surveys (MEDITS) from
+1999-2021 for the Western Mediterranean sub-basin (Fig. 3.7.1). This region covers from the
+Strait of Gibraltar to the Strait of Sicily and includes 9 fisheries management areas (i.e.,
+Geographical Sub-Areas, GSA) assessed by the General Fisheries Commission for the
+Mediterranean (GFCM). MEDITS data collection follows standardized protocols that account
+for gears, sampling scheme and biological procedures for data collection; details in Spedicato
+et al. 2019, 2024. A total of 12.666 locations were sampled over 23 years in pre-defined
+locations following a depth-stratified scheme. This study focuses only on the presence and
+abundance (individuals · km-2) of main demersal macrofaunal species and, therefore we only
+consider fish (Elasmobranchii and Teleostei), cephalopods (Cephalopoda) and decapod
+crustaceans (Malacostraca) groups. </t>
+  </si>
+  <si>
+    <t>We compile information on different
+functional traits from FishBase (Froese &amp; Pauly, 2023; Boettinger, 2012), SeaLifeBase
+(Palomares and Pauly, 2023) and primary literature (see details Spedicato et al. 2024).
+Continues traits include body length, life span, larval and juvenile development, vertical
+biological zone, depth range and temperature preferences and diet as categorical traits. For
+the feasibility of the statistical analyses, we only selected the species that fullfil with the
+following criteria: i) occurred in at least 1% of the hauls (approximately 200 occurrences)
+across the complete time series and, ii) information on life-history and ecological traits was
+available. Final species selection accounts for a total of 191 species, including 146 fish, 24
+cephalopods and 21 crustaceans.</t>
+  </si>
+  <si>
+    <t>HMSC was used to model demersal communities using the hurdle approach by modeling
+independently presence-absence (PA model) from abundance data (AB model), using probit
+and log-linear regression, respectively. Both models used the same setup and
+parameterization, assuming the default prior distribution, and including as linear fixed effects
+all the environmental variables (substrate, SST, botTemp, so, botso, chl, FPI). We included
+second-order polynomial terms for temperature and salinity variables, since many species
+may display optimum ranges in their environmental niches. The rest of the explanatory
+variables were assumed to display linear relationship. As random effects, we included the year
+of the survey and a fixed hexagonal grid of 0.042° as spatial units (N=1121; instead of haul locations) to reduce the complexity of the spatial structure. Models were fitted independently
+with the Markov chain Monte Carlo (MCMC) method implemented in ‘Hmsc’ R-package
+(Tikhonov et al. 2020). Each of the four MCMC included 250 samples with a thinning of 100
+with the first 12.500 discarded as burn in, therefore, running 37.500 iterations and returning
+1000 posterior samples in total for each model. Convergence was assessed with the Gelman-
+Rubin potential scale reduction factor (psrf; Gelman and Rubin 1992). Explanatory power was
+estimated using root mean square error (RMSE), as well as the area under the curve (AUC;
+Pearce &amp; Ferrier 2000) and the coefficient of discrimination (Tjur R2; Tjur 2009) values for
+presence-absence model and, using R2 in the abundance model. To compute predictive
+power, 4-fold cross-validation was performed in each of the models. Final predictions were
+the product of the two model predictions, as an estimate of species abundance conditioned
+on presence over the 0.042° spatial grid. Prior computing final predictions, species presence
+(i.e., threshold between zero and one values) was set using a species-specific threshold that
+maximize the Percentage of Correct Classification (PCC) using “PresenceAbsence” R package
+(Manel et al. 2001, Wilson et al. 2004, Freeman and Moisen 2008). Final predictions were used
+to compute a suite of biodiversity indicators including taxonomic and functional richness,
+evenness and dispersion.</t>
   </si>
 </sst>
 </file>
@@ -794,12 +1199,146 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A5808B4-DED8-4038-83E2-89CC5F8B5437}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <cols>
+    <col min="1" max="1" width="32.08984375" customWidth="1"/>
+    <col min="2" max="2" width="134.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="162.25" x14ac:dyDescent="0.75">
+      <c r="A3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="147.5" x14ac:dyDescent="0.75">
+      <c r="A4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="206.5" x14ac:dyDescent="0.75">
+      <c r="A5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="383.5" x14ac:dyDescent="0.75">
+      <c r="A6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A7" t="s">
+        <v>76</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{532B325C-EC70-401B-9B81-E90568F4AE5E}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <cols>
+    <col min="1" max="1" width="15.08984375" customWidth="1"/>
+    <col min="2" max="2" width="197.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="28.75" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="409.5" x14ac:dyDescent="0.75">
+      <c r="A3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="132.75" x14ac:dyDescent="0.75">
+      <c r="A4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="354" x14ac:dyDescent="0.75">
+      <c r="A5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="409.5" x14ac:dyDescent="0.75">
+      <c r="A6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A7" t="s">
+        <v>76</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCDFC4F4-DA9B-4676-B4E9-27438403FC6D}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="14.08984375" customWidth="1"/>
+    <col min="1" max="1" width="14.1328125" customWidth="1"/>
     <col min="2" max="2" width="110.40625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -909,7 +1448,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7534530D-A73A-4258-8656-ECA9512F2226}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
     <col min="1" max="1" width="19.40625" bestFit="1" customWidth="1"/>
@@ -945,7 +1484,31 @@
         <v>49</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A5" t="s">
         <v>66</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A7" t="s">
+        <v>68</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1036,7 +1599,7 @@
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="2" max="2" width="95.6328125" customWidth="1"/>
+    <col min="2" max="2" width="95.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.75">
@@ -1047,12 +1610,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="73.75" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" ht="221.25" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
         <v>56</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="103.25" x14ac:dyDescent="0.75">
@@ -1120,4 +1683,137 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56BED128-4941-403A-8B14-BE1B70CB049C}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <cols>
+    <col min="2" max="2" width="149.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="29.5" x14ac:dyDescent="0.75">
+      <c r="A2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="409.5" x14ac:dyDescent="0.75">
+      <c r="A4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="132.75" x14ac:dyDescent="0.75">
+      <c r="A5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="409.5" x14ac:dyDescent="0.75">
+      <c r="A6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A7" t="s">
+        <v>76</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19212195-0A71-4EBF-B930-11848C857DE8}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <cols>
+    <col min="1" max="1" width="17.6328125" customWidth="1"/>
+    <col min="2" max="2" width="149.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="58.75" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="295" x14ac:dyDescent="0.75">
+      <c r="A3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="206.5" x14ac:dyDescent="0.75">
+      <c r="A4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="368.75" x14ac:dyDescent="0.75">
+      <c r="A5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="409.5" x14ac:dyDescent="0.75">
+      <c r="A6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+      <c r="A7" t="s">
+        <v>76</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
commit final files and edits
</commit_message>
<xml_diff>
--- a/data-raw/project_texts.xlsx
+++ b/data-raw/project_texts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\neilm\Projects\b_useful\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB493EBE-2960-4678-927A-D484D3241616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BFC7A0B-9CF0-44AA-BA61-066BC4D1ED86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" firstSheet="6" activeTab="9" xr2:uid="{B3A1738F-4730-4C3D-B31B-830F2610B29E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="6" activeTab="10" xr2:uid="{B3A1738F-4730-4C3D-B31B-830F2610B29E}"/>
   </bookViews>
   <sheets>
     <sheet name="landing_page" sheetId="1" r:id="rId1"/>
@@ -528,165 +528,6 @@
     <t>Walter Zupa, Antonella Consiglio, Matteo Chiarini, Maria Teresa Spedicato</t>
   </si>
   <si>
-    <t>Data on the occurrence and abundance of demersal species were obtained from the
-Mediterranean International Bottom Trawl Survey MEDITS (Bertrand et al., 2002; Spedicato
-et al., 2019) conducted annually from May to July since 1994, recently under the EU Data
-Collection Framework (DCF; EU, (EU) 2017/1004). The survey applies a stratified random
-sampling scheme, with haul allocation proportional to the surface area of 5 depth strata
-(covering the bathymetrical range from 10m to 800m). The analyses focused on nine
-Geographical Sub-Areas (GSAs; GFCM, 2009) of the Central and Eastern Mediterranean Sea,
-specifically: GSA 15 (Malta), GSA 16 (Southern Sicily), GSA 17 (Northern Adriatic Sea), GSA 18
-(Southern Adriatic Sea), GSA 19 (Western Ionian Sea), GSA 20 (Eastern Ionian Sea), GSA 22
-(Aegean Sea), GSA 23 (Crete), and GSA 25 (Cyprus), as illustrated in Figure 3.6.1. The selected
-spatial domain covers approximately 378,852 km2 with, on average, about 577 sampling
-stations per year. The selected temporal range for the analysis spans from 1999 to 2021 to
-provide comprehensive coverage of environmental drivers used in modeling. Although the
-MEDITS survey has been conducted regularly on an annual basis, some gaps in temporal
-continuity occurred in some GSAs, such as GSA 15 and GSA 25, where sampling began in 2005,
-and some annual gaps between 2009 and 2013 in GSAs 20, 22, and 23. The survey is conducted
-in each GSA using the GOC 73 trawl gear, which is equipped with a 20 mm stretched mesh
-codend (Bertrand et al., 2002; Spedicato et al., 2019), allowing for the capture of small-sized
-individuals. Once onboard, all specimens exceeding 1 cm in size are taxonomically identified,
-and both their number and total biomass are recorded. This procedure generates a consistent
-dataset that supports the calculation of standardized abundance indices (expressed as N/km²)
-across hauls. &lt;br&gt;To ensure the quality of data used for the analysis, a multiple and comprehensive data
-validation procedure was applied on MEDITS data using the R package RoME
-(https://github.com/COISPA/RoME), routinely adopted by the MEDITS coordination group
-and embedded in the newly developed Med&amp;BS RDBFIS regional database in the
-Mediterranean (https://medbsrdb.eu/), extensively checked by experts in the QualiTrain EU
-project (EASME/EMFF/2020/OP/021). This process allows the users to easily identify the
-presence of inconsistencies in the source data, such as haul position, taxonomic classification,
-measure units, number of individuals caught, and their relative weights, which could likely
-affect the results of the modeling analysis. Consequently, data correction procedures were
-carried out, particularly oriented to address issues linked to the estimation of the sampling
-positions and of the abundance indices at the species level. To define the species pool used in
-the HMSC modeling, we calculated the occurrence and frequency of all taxa recorded in the
-catches of the dataset across all hauls of the geographical domain of the study. Species
-belonging to fish (A), decapod crustaceans (B), and cephalopods (C) were retained. The initial
-MEDITS dataset covering the study area comprised a total of 599 taxa, including 371 fish
-species (of which 321 were teleosts and 50 elasmobranchs) alongside 47 cephalopod species
-and 181 crustacean taxa. For the main analysis, we selected species with frequency of
-occurrence &gt; 1%, resulting in a final list of 184 taxa. A subsequent screening based on the
-availability of trait information led to a further reduction of the dataset, retaining 158 taxa for
-modeling purposes (120 fish, 18 crustaceans, and 20 cephalopods).</t>
-  </si>
-  <si>
-    <t>In parallel with the species occurrence and abundance, a comprehensive life-history trait
-database was developed ad hoc, as reported in the Deliverable D2.2 (https://buseful.
-eu/library/deliverables/; Spedicato et al., 2024), including 15 different traits (9
-continuous and 6 categorical). Trait databases for crustaceans and cephalopods were
-compiled, drawing primarily from SeaLifeBase (Palomares &amp; Pauly, 2022), while for fish, the
-trait dataset was assembled mostly based on Beukhof et al. (2019) complemented by FishBase
-(Froese, 2005), and through phylogenetic imputation using the R package phylosem (Thorson
-&amp; van der Bijl, 2023). The traits database was finally composed of references for 363 fish taxa,
-72 crustaceans, and 62 cephalopods.</t>
-  </si>
-  <si>
-    <t>To characterize the environmental conditions at each
-sampling location, we extracted a comprehensive set of physical and biogeochemical variables
-from the Copernicus Marine Environment Monitoring Service (CMEMS)
-(https://marine.copernicus.eu) using the reanalysis products with a monthly temporal
-resolution and a spatial resolution of 1/24° (~0.042°). Specifically, we used the product
-MEDSEA_MULTIYEAR_PHY_006_004 (Escudier et al., 2021) to retrieve sea surface and bottom
-temperature (°C) and salinity (PSU), and the product MEDSEA_MULTIYEAR_BGC_006_008
-(Cossarini et al., 2021) for surface chlorophyll-a concentration (mg m⁻³), net primary
-production (mmol N m⁻³ day⁻¹), nitrate (mmol N m⁻³), phosphate (mmol P m⁻³), dissolved
-oxygen (mmol O₂ m⁻³), and phytoplankton concentration (mmol N m⁻³). In addition, current
-velocity data were used to derive eastward and northward components of horizontal
-circulation. Furthermore, seabed substrate classification was retrieved from EMODnet
-Geology (European Marine Observation and Data network; www.emodnet-geology.eu), using
-the EUSeaMap 2023 Broad-Scale Predictive Habitat Map for Europe product (Vasquez et al.,
-2023), whereas bathymetry product tiles (EMODnet Bathymetry portal,
-http://www.emodnet-bathymetry.eu) were used to retrieve depth information. In addition,
-other pressure drivers were explored in the models’ setup, such as the gravity index (Cinner
-et al., 2018), the fishing pressure index (FPI) estimated with the application of multi-criteria decision analysis (MCDA) (Kavadas et al., 2015) and the fishing effort information provided by
-DCF Fisheries Dependent Information (FDI), spatially disaggregated by means of a fishing
-footprint derived from Global Fishing Watch (GFW). Before the model fitting, collinearity
-among environmental covariates was assessed using Pearson’s correlation matrix (Annex 6,
-Figure S1). Only predictors with pairwise correlation coefficients below 0.7 were retained as a
-conservative rule of thumb (Dormann et al., 2013), to minimize redundancy and avoid strong
-collinearity.</t>
-  </si>
-  <si>
-    <t>The HMSC framework was employed to model and investigate the drivers and community
-responses acting on the Mediterranean demersal communities through the R package Hmsc
-version 3.3-4 (Ovaskainen et al., 2017; Tikhonov et al., 2020). Due to the zero-inflated
-distribution of the data, a hurdle approach involving two separate models was adopted: a
-presence–absence model (occurrence) based on a probit distribution combined with an
-abundance conditional on presence model (abundance model). The abundance models were
-tested using different distributions, although the normal distribution was retained as it
-provided the best fitting performance. Two different hurdle models were finally produced:
-one using the whole time series (WTS), spanning from 1999 to 2021, and another using a
-shortened time series (2012–2021) that allowed the inclusion of fishing effort (FE) derived
-from DCF FDI data, spatially disaggregated using the GFW fishing footprint, which was not
-tested in the WTS models. Each model included both random and fixed effects. The former
-was selected to account for the spatial and temporal variations (by means of the inclusion of
-the grid cells and the year effects) not directly incorporated as fixed components. As fixed
-effects, bottom temperature, bottom salinity, depth, and chlorophyll-a concentration were
-finally retained in both WTS and FE models. To account for potential non-linear species–
-environment relationships, for both models, a second-degree polynomial function was
-applied to depth, for the occurrence sub-models, and extended to all other environmental
-covariates for the abundance models, except for chlorophyll-a. Chlorophyll-a concentration
-and fishing effort (for the FE model) were log-transformed to reduce variability and to improve
-the linearity of their relationship with the species response.&lt;br&gt;
-To account for interspecific variation in ecological strategies to environmental variables and
-reduce computational performance, a set of biologically meaningful traits was selected and
-incorporated into the models. The retained traits included maximum length, longevity, depth
-preference, temperature preference, and trophic level, and were applied consistently across
-taxonomic groups, including fishes, crustaceans, and cephalopods. These traits were selected
-based on their ecological relevance in structuring demersal communities and mediating
-responses to external pressure drivers. Maximum body length and longevity are key life history
-traits associated with species' reproductive output, population turnover, and
-sensitivity to exploitation (Hiddink et al., 2019; Quesne &amp; Jennings, 2012). Depth and
-temperature preferences reflect species’ niche and are critical traits determining the spatial
-distribution (Polo et al., 2025; Stuart-Smith et al., 2015). Trophic level situates species within
-the food web and is important for understanding predator–prey interactions (Romanuk et al.,
-2011). Four Markov Chain Monte Carlo (MCMC) chains were run, each drawing 250 posterior
-samples, for a total of 1000 samples. Thinning intervals were thus adjusted for each model
-individually to optimise convergence diagnostics, while ensuring computational feasibility, finally adopting a thinning interval of 2000. To ensure that the chains reached their stationary
-distribution before posterior sampling, a burn-in phase of 250,000 iterations (transients) was
-applied. As a result, each chain executed a total of 750,000 iterations (250,000 burn-in +
-500,000 sampling), yielding an overall computational effort of 3 million iterations across the
-four chains. This modeling setup adheres to widely accepted practices in Bayesian inference,
-where sufficient burn-in and thinning are essential to reduce the impact of initialisation and
-autocorrelation (Geyer, 2011; Margossian et al., 2023). Convergence of the MCMC was
-assessed by evaluating the Potential Scale Reduction Factor (PSRF; Gelman &amp; Rubin, 1992) of
-model parameters, with convergence considered satisfactory when the mean PSRF values do
-not exceed 1.1 (Tikhonov et al., 2020). Convergence of the MCMC chains was further assessed
-using the Geweke diagnostic (Geweke, 1992) for each model parameter, and convergence was
-considered satisfactory when |z| &lt; 1.96. The model performances were evaluated as both
-explanatory and predictive power through a 4-fold cross-validation. In each fold, the models
-were trained on 75% of the data and tested on the remaining 25%, iteratively covering the
-entire dataset. To quantify model performance, a set of complementary metrics was used,
-tailored to the nature of the models. For the occurrence model the following metrics were
-used: the area under the operating characteristic curve (AUC) and Tjur’s coefficient of
-discrimination (Tjur R²), a robust measure for binary response models that reflects the
-difference in predicted probabilities between observed presences and absences (Tjur, 2009).
-For the abundance (conditional-on-presence) model, the R² was used instead, while in both
-models the root mean square error (RMSE) was estimated as an indicator of the average
-deviation between observed and predicted values. All the statistical analyses were conducted
-in R software version 4.4.1 (R Core Team, 2024). The model runs and the cross-validation were
-performed on the DRAGO high-performance computing (HPC) cluster hosted by the Consejo
-Superior de Investigaciones Científicas (CSIC), exploiting the HMSC-HPC implementation using
-NVIDIA A100 40GB GPUs. For each cross-validation fold and MCMC chain, independent jobs
-were launched in parallel, allowing efficient scaling of the workload across the cluster.
-Based on the models’ predictions a set of biodiversity indicators was estimated. Taxonomic
-richness was assessed as the total number of species present at each site, considering only
-those species with an occurrence probability equal to or greater than 0.2. This threshold was
-chosen to avoid excluding rare species that typically exhibit low predicted occurrence
-probabilities, aligning with other studies that favor more inclusive thresholds (Chou et al.,
-2020; Linhoss and Mickle, 2022). The Shannon diversity index (H') was calculated using the R
-package vegan. Pielou’s evenness index (J') was computed as the ratio between the Shannon
-index and the natural logarithm of species richness. To quantify functional diversity, we
-calculated functional richness (FRic) and functional evenness (FEve) by constructing a
-multidimensional trait space. This was achieved through a Principal Coordinates Analysis
-(PCoA) based on Gower distances between species traits (Legendre and Legendre, 1998).
-These metrics describe the extent to which species occupy the available functional trait space
-within the community, and the uniformity of biomass distribution across that space (Mouillot
-et al., 2013). We retained the first three Principal Coordinates (PCs), with a cumulative
-explained variance of 83%.</t>
-  </si>
-  <si>
     <t>Patricia Puerta, Alicia Gran, Manuel Hidalgo</t>
   </si>
   <si>
@@ -756,6 +597,90 @@
 (Manel et al. 2001, Wilson et al. 2004, Freeman and Moisen 2008). Final predictions were used
 to compute a suite of biodiversity indicators including taxonomic and functional richness,
 evenness and dispersion.</t>
+  </si>
+  <si>
+    <t>Data on the occurrence and abundance of demersal species were obtained from the Mediterranean International Bottom Trawl Survey MEDITS (Bertrand et al., 2002; Spedicato et al., 2019) conducted annually from May to July since 1994, recently under the EU Data Collection Framework (DCF; EU, (EU) 2017/1004). The survey applies a stratified random sampling scheme, with haul allocation proportional to the surface area of 5 depth strata (covering the bathymetrical range from 10m to 800m). The analyses focused on nine Geographical Sub-Areas (GSAs; GFCM, 2009) of the Central and Eastern Mediterranean Sea, specifically: GSA 15 (Malta), GSA 16 (Southern Sicily), GSA 17 (Northern Adriatic Sea), GSA 18 (Southern Adriatic Sea), GSA 19 (Western Ionian Sea), GSA 20 (Eastern Ionian Sea), GSA 22 (Aegean Sea), GSA 23 (Crete), and GSA 25 (Cyprus), as illustrated in Figure 3.6.1. The selected spatial domain covers approximately 378,852 km2 with, on average, about 577 sampling stations per year. The selected temporal range for the analysis spans from 2012 to 2021 to provide comprehensive coverage of environmental drivers used in modelling, particularly the available AIS data of fishing effort. Although the MEDITS survey has been conducted regularly on an annual basis, some gaps in temporal continuity occurred in some GSAs, such as some annual gaps between 2009 and 2013 in GSAs 20, 22, and 23. The survey is conducted in each GSA using the GOC 73 trawl gear, which is equipped with a 20 mm stretched mesh codend (Bertrand et al., 2002; Spedicato et al., 2019), allowing for the capture of small-sized individuals. Once onboard, all specimens exceeding 1 cm in size are taxonomically identified, and both their number and total biomass are recorded. This procedure generates a consistent dataset that supports the calculation of standardized abundance indices (expressed as N/km²) across hauls.
+&lt;br&gt;&lt;br&gt;
+To ensure the quality of data used for the analysis, a multiple and comprehensive data validation procedure was applied on MEDITS data using the R package RoME (https://github.com/COISPA/RoME), routinely adopted by the MEDITS coordination group and embedded in the newly developed Med&amp;BS RDBFIS regional database in the Mediterranean (https://medbsrdb.eu/), extensively checked by experts in the QualiTrain EU project (EASME/EMFF/2020/OP/021). This process allows the users to easily identify the presence of inconsistencies in the source data, such as haul position, taxonomic classification, measure units, number of individuals caught, and their relative weights, which could likely affect the results of the modeling analysis. Consequently, data correction procedures were carried out, particularly oriented to address issues linked to the estimation of the sampling positions and of the abundance indices at the species level. To define the species pool used in the HMSC modeling, we calculated the occurrence and frequency of all taxa recorded in the catches of the dataset across all hauls of the geographical domain of the study. Species belonging to fish (A), decapod crustaceans (B), and cephalopods (C) were retained. The initial MEDITS dataset covering the study area comprised a total of 599 taxa, including 371 fish species (of which 321 were teleosts and 50 elasmobranchs) alongside 47 cephalopod species and 181 crustacean taxa. For the main analysis, we selected species with frequency of occurrence &gt; 1%, resulting in a final list of 184 taxa. A subsequent screening based on the availability of trait information led to a further reduction of the dataset, retaining 158 taxa for modeling purposes (120 fish, 18 crustaceans, and 20 cephalopods).</t>
+  </si>
+  <si>
+    <t>In parallel with the species occurrence and abundance, a comprehensive life-history trait database was developed ad hoc, as reported in the Deliverable D2.2 (https://buseful. eu/library/deliverables/; Spedicato et al., 2024), including 15 different traits (9 continuous and 6 categorical). Trait databases for crustaceans and cephalopods were compiled, drawing primarily from SeaLifeBase (Palomares &amp; Pauly, 2022), while for fish, the trait dataset was assembled mostly based on Beukhof et al. (2019) complemented by FishBase (Froese, 2005), and through phylogenetic imputation using the R package phylosem (Thorson &amp; van der Bijl, 2023). The traits database was finally composed of references for 363 fish taxa, 72 crustaceans, and 62 cephalopods.</t>
+  </si>
+  <si>
+    <t>To characterize the environmental conditions at each sampling location, we extracted a comprehensive set of physical and biogeochemical variables to be tested in the modelling phase, including MEDSEA_MULTIYEAR_PHY_006_004 product (Escudier et al., 2021) to retrieve sea surface and bottom temperature (°C) and salinity (PSU), and the product MEDSEA_MULTIYEAR_BGC_006_008 (Cossarini et al., 2021) for surface chlorophyll-a concentration (mg m⁻³), net primary production (mmol N m⁻³ day⁻¹), nitrate (mmol N m⁻³), phosphate (mmol P m⁻³), dissolved oxygen (mmol O₂ m⁻³), and phytoplankton concentration (mmol N m⁻³). In addition, current velocity data were used to derive eastward and northward components of horizontal circulation. Seabed substrate classification was retrieved from EMODnet Geology (European Marine Observation and Data network; www.emodnet-geology.eu), using the EUSeaMap 2023 Broad-Scale Predictive Habitat Map for Europe product (Vasquez et al., 2021), whereas bathymetry product tiles (EMODnet Bathymetry portal, http://www.emodnet-bathymetry.eu) were used to retrieve depth information. In addition, fishing effort driver was included in the models’ setup using the fishing effort information provided by DCF Fisheries Dependent Information (FDI), spatially disaggregated by means of a fishing footprint derived from Global Fishing Watch (GFW). Before the model fitting, collinearity among environmental covariates was assessed using Pearson’s correlation matrix (Annex 6, Figure S1).
+&lt;br&gt;&lt;br&gt;
+Future projections based on climatic variations were obtained by using the environmental predictors from the dataset of Copernicus Climate Change Service, using the POLCOMS/NEMO-ERSEM model (Copernicus Climate Change Service, 2020) , using the business-as-usual scenario RCP8.5, which assumes that greenhouse gas emissions continue to rise throughout the century (Kay, 2020). Because the environmental covariates used to fit the species–environment relationships and those used in the climate projections came from different data sources, a mean bias correction (delta correction) was applied to harmonise offsets between datasets and bring the projected climatic data onto the same scale as the historical baseline (Kuehn, 2023).</t>
+  </si>
+  <si>
+    <t>The HMSC framework was employed to model and investigate the drivers and community responses acting on the Mediterranean demersal communities through the R package Hmsc version 3.3-4 (Ovaskainen et al., 2017; Tikhonov et al., 2020a). Due to the zero-inflated distribution of the data, a hurdle approach involving two separate models was adopted: a presence–absence model (occurrence) based on a probit distribution combined with an abundance conditional on presence model (abundance model). The abundance models were tested using different distributions, although the normal distribution was retained as it provided the best fitting performance. The hurdle models was finally trained spanning from 2012 to 2021. The model included both random and fixed effects. The former was selected to account for the spatial and temporal variations (by means of the inclusion of the grid cells and the year effects) not directly incorporated as fixed components.
+&lt;br&gt;&lt;br&gt;
+Only predictors with pairwise correlation coefficients below 0.7 were retained as a conservative rule of thumb (Dormann et al., 2013) , to minimize redundancy and avoid strong collinearity. As fixed effects, bottom temperature, bottom salinity, depth, and chlorophyll-a concentration were finally retained in the model. To account for potential non-linear species– environment relationships a second-degree polynomial function was applied to depth, for the occurrence sub-models, and extended to all other environmental covariates for the abundance models, except for chlorophyll-a. Chlorophyll-a concentration and fishing effort (for the FE model) were log-transformed to reduce variability and to improve the linearity of their relationship with the species response.
+&lt;br&gt;&lt;br&gt;
+To account for interspecific variation in ecological strategies to environmental variables and reduce computational performance, a set of biologically meaningful traits was selected and incorporated into the models. The retained traits included maximum length, longevity, depth preference, temperature preference, and trophic level, and were applied consistently across taxonomic groups, including fishes, crustaceans, and cephalopods. These traits were selected based on their ecological relevance in structuring demersal communities and mediating responses to external pressure drivers. Maximum body length and longevity are key life history traits associated with species' reproductive output, population turnover, and sensitivity to exploitation (Hiddink et al., 2019; Le Quesne &amp; Jennings, 2012) . Depth and temperature preferences reflect species’ niche and are critical traits determining the spatial distribution (Polo et al., 2025; Stuart-Smith et al., 2015). Trophic level allocates species within the food web and is important for understanding predator–prey interactions (Romanuk et al., 2011). Four Markov Chain Monte Carlo (MCMC) chains were run, each drawing 250 posterior samples, for a total of 1000 samples. Thinning intervals were thus adjusted for each model individually to optimise convergence diagnostics, while ensuring computational feasibility, finally adopting a thinning interval of 2000. To ensure that the chains reached their stationary distribution before posterior sampling, a burn-in phase of 250,000 iterations (transients) was applied. As a result, each chain executed a total of 750,000 iterations (250,000 burn-in + 500,000 sampling), yielding an overall computational effort of 3 million iterations across the four chains. This modeling setup adheres to widely accepted practices in Bayesian inference, where sufficient burn-in and thinning are essential to reduce the impact of initialisation and autocorrelation (Jambeck et al., 2015; Margossian et al., 2023). Convergence of the MCMC was assessed by evaluating the Potential Scale Reduction Factor (PSRF; Gelman &amp; Rubin, 1992) of model parameters, with convergence considered satisfactory when the mean PSRF values do not exceed 1.1 (Tikhonov et al., 2020b). Convergence of the MCMC chains was further assessed using the Geweke diagnostic (Geweke, 1992) for each model parameter, and convergence was considered satisfactory when |z| &lt; 1.96. The model performances were evaluated as both explanatory and predictive power through a 4-fold cross-validation. In each fold, the models were trained on 75% of the data and tested on the remaining 25%, iteratively covering the entire dataset. To quantify model performance, a set of complementary metrics was used, tailored to the nature of the models. For the occurrence model the following metrics were used: the area under the operating characteristic curve (AUC) and Tjur’s coefficient of discrimination (Tjur R²), a robust measure for binary response models that reflects the difference in predicted probabilities between observed presences and absences (Tjur, 2009). For the abundance (conditional-on-presence) model, the R² was used instead, while in both models the root mean square error (RMSE) was estimated as an indicator of the average deviation between observed and predicted values. All the statistical analyses were conducted in R software version 4.4.1 (R Core Team, 2024). The model runs and the cross-validation were performed on the DRAG+B18O high-performance computing (HPC) cluster hosted by the Consejo Superior de Investigaciones Científicas (CSIC), exploiting the HMSC-HPC implementation using NVIDIA A100 40GB GPUs. For each cross-validation fold and MCMC chain, independent jobs were launched in parallel, allowing efficient scaling of the workload across the cluster.
+&lt;br&gt;&lt;br&gt;
+MCMC convergence diagnostics indicated robust convergence for both the occurrence and abundance sub-models. the mean PSRF values for the beta parameter of the occurrence and abundance were 1.005 and 1.029, respectively, and 1.006 for the abundance sub-model, and 1.003 for the occurrence model for the gamma parameter. Despite the presence of a few outlier parameters, the overall means remained well below the commonly accepted threshold of 1.1, confirming good chain mixing. Effective Sample Size (ESS) values were also consistently high, with mean values exceeding 995 for all parameter groups, indicating highly efficient sampling and low autocorrelation. These results were further supported by the Geweke diagnostic, with 91.5% and 91.3% of the parameters passing the test in the occurrence and abundance sub-models. The combination of diagnostics provides strong evidence of reliable posterior estimation.
+&lt;br&gt;&lt;br&gt;
+In terms of models’ explanatory and predictive capacity the occurrence model showed excellent discriminatory ability, with AUC values close or equal to 0.9 (explanatory power = 0.9; predictive power = 0.895), and consistent Tjur’s R² and RMSE values (0.3 and 0.24 respectively). The near-identical performance metrics between the explanatory and predictive assessments further highlight that the cross-validation procedure demonstrated the robustness of the models’ predictive capabilities, supporting the idea that the model is generalizable and not overfitted to the dataset.
+&lt;br&gt;&lt;br&gt;
+Taxonomic richness was calculated as the number of species predicted to be present at each site. Species presence was determined using species-specific probability thresholds estimated from hindcast predictions and observed presence–absence data. For each species, the threshold maximizing the overall proportion of correctly classified presences and absences (percent correctly classified, PCC) based on the confusion matrix was selected (Cantor et al., 1999; Freeman &amp; Moisen, 2008; Manel et al., 2001) .
+&lt;br&gt;&lt;br&gt;
+The Shannon diversity index (H') was calculated using the R package vegan. Pielou’s evenness index (J') was computed as the ratio between the Shannon index and the natural logarithm of species richness. To quantify functional diversity, we calculated functional richness (FRic) and functional evenness (FEve) by constructing a multidimensional trait space. This was achieved through a Principal Coordinates Analysis (PCoA) based on Gower distances between species traits (Legendre &amp; Legendre, 1998) . These metrics describe the extent to which species occupy the available functional trait space within the community, and the uniformity of biomass distribution across that space (Mouillot et al., 2013) . Three Principal Coordinate axes were retained based on the quality of the resulting functional space using the scaled mean absolute deviation criterion; together, these axes accounted for 71.6% of the total positive PCoA inertia.&lt;br&gt;&lt;br&gt;&lt;h2&gt;References&lt;/h2&gt;&lt;p&gt;Bertrand, J. A., De Sola, L. G., Papaconstantinou, C., Relini, G., &amp;amp; Souplet, A. (2002). The general specifications of the MEDITS surveys. &lt;em&gt;Scientia Marina, 66&lt;/em&gt;(S2). &lt;a href="https://doi.org/10.3989/scimar.2002.66s29"&gt;https://doi.org/10.3989/scimar.2002.66s29&lt;/a&gt;
+&lt;br&gt;&lt;br&gt;
+Beukhof, E., Dencker, T. S., Palomares, M. L. D., &amp;amp; Maureaud, A. (2019). A trait collection of marine fish species from North Atlantic and Northeast Pacific continental shelf seas. &lt;em&gt;Pangaea, 1&lt;/em&gt;, 12.
+&lt;br&gt;&lt;br&gt;
+Cantor, S. B., Sun, C. C., Tortolero-Luna, G., Richards-Kortum, R., &amp;amp; Follen, M. (1999). A comparison of C/B ratios from studies using receiver operating characteristic curve analysis. &lt;em&gt;Journal of Clinical Epidemiology, 52&lt;/em&gt;(9), 885–892.
+&lt;br&gt;&lt;br&gt;
+Copernicus Climate Change Service. (2020). Marine biogeochemistry data for the Northwest European Shelf and Mediterranean Sea from 2006 up to 2100 derived from climate projections. &lt;em&gt;Copernicus Climate Change Service (C3S) Climate Data Store (CDS)&lt;/em&gt;. &lt;a href="https://doi.org/10.24381/cds.dcc9295c"&gt;https://doi.org/10.24381/cds.dcc9295c&lt;/a&gt;
+&lt;br&gt;&lt;br&gt;
+Cossarini, G., Feudale, L., Teruzzi, A., Bolzon, G., Coidessa, G., Solidoro, C., Di Biagio, V., Amadio, C., Lazzari, P., &amp;amp; Brosich, A. (2021). High-resolution reanalysis of the Mediterranean Sea biogeochemistry (1999–2019). &lt;em&gt;Frontiers in Marine Science, 8&lt;/em&gt;, 741486. &lt;a href="https://doi.org/10.3389/fmars.2021.741486"&gt;https://doi.org/10.3389/fmars.2021.741486&lt;/a&gt;
+&lt;br&gt;&lt;br&gt;
+Dormann, C. F., Elith, J., Bacher, S., Buchmann, C., Carl, G., Carré, G., Marquéz, J. R. G., Gruber, B., Lafourcade, B., Leitão, P. J., &amp;amp; others. (2013). Collinearity: A review of methods to deal with it and a simulation study evaluating their performance. &lt;em&gt;Ecography, 36&lt;/em&gt;(1), 27–46.
+&lt;br&gt;&lt;br&gt;
+Escudier, R., Clementi, E., Cipollone, A., Pistoia, J., Drudi, M., Grandi, A., Lyubartsev, V., Lecci, R., Aydogdu, A., &amp;amp; Delrosso, D. (2021). A high resolution reanalysis for the Mediterranean Sea. &lt;em&gt;Frontiers in Earth Science, 9&lt;/em&gt;, 702285. &lt;a href="https://doi.org/10.3389/feart.2021.702285"&gt;https://doi.org/10.3389/feart.2021.702285&lt;/a&gt;
+&lt;br&gt;&lt;br&gt;
+Freeman, E. A., &amp;amp; Moisen, G. (2008). PresenceAbsence: An R package for presence absence analysis. &lt;em&gt;Journal of Statistical Software, 23&lt;/em&gt;, 1–31.
+&lt;br&gt;&lt;br&gt;
+Froese, R. (2005). &lt;em&gt;FishBase&lt;/em&gt;. World Wide Web electronic publication. &lt;a href="https://www.fishbase.org/"&gt;www.fishbase.org&lt;/a&gt;.
+&lt;br&gt;&lt;br&gt;
+Gelman, A., &amp;amp; Rubin, D. B. (1992). Inference from iterative simulation using multiple sequences. &lt;em&gt;Statistical Science, 7&lt;/em&gt;(4), 457–472.
+&lt;br&gt;&lt;br&gt;
+Geweke, J. (1992). Evaluating the accuracy of sampling-based approaches to the calculations of posterior moments. &lt;em&gt;Bayesian Statistics, 4&lt;/em&gt;, 641–649.
+&lt;br&gt;&lt;br&gt;
+Hiddink, J. G., Jennings, S., Sciberras, M., Bolam, S. G., Cambiè, G., McConnaughey, R. A., Mazor, T., Hilborn, R., Collie, J. S., &amp;amp; Pitcher, C. R. (2019). Assessing bottom trawling impacts based on the longevity of benthic invertebrates. &lt;em&gt;Journal of Applied Ecology, 56&lt;/em&gt;(5), 1075–1084.
+&lt;br&gt;&lt;br&gt;
+Jambeck, J. R., Geyer, R., Wilcox, C., Siegler, T. R., Perryman, M., Andrady, A., Narayan, R., &amp;amp; Law, K. L. (2015). Plastic waste inputs from land into the ocean. &lt;em&gt;Science, 347&lt;/em&gt;(6223), 768–771. &lt;a href="https://doi.org/10.1126/science.1260352"&gt;https://doi.org/10.1126/science.1260352&lt;/a&gt;
+&lt;br&gt;&lt;br&gt;
+Kay, S. (2020). Marine biogeochemistry data for the Northwest European Shelf and Mediterranean Sea from 2006 up to 2100 derived from climate projections. &lt;em&gt;Copernicus Climate Change Service (C3S) Climate Data Store (CDS)&lt;/em&gt;. &lt;a href="https://doi.org/10.24381/cds.dcc9295c"&gt;https://doi.org/10.24381/cds.dcc9295c&lt;/a&gt;
+&lt;br&gt;&lt;br&gt;
+Kuehn, B. (2023). Tutorial - Ways to bias correct climate projections. &lt;em&gt;figshare&lt;/em&gt;. &lt;a href="https://doi.org/10.6084/m9.figshare.23514618.v1"&gt;https://doi.org/10.6084/m9.figshare.23514618.v1&lt;/a&gt;
+&lt;br&gt;&lt;br&gt;
+Le Quesne, W. J. F., &amp;amp; Jennings, S. (2012). Predicting species vulnerability with minimal data to support rapid risk assessment of fishing impacts on biodiversity. &lt;em&gt;Journal of Applied Ecology, 49&lt;/em&gt;(1), 20–28. &lt;a href="https://doi.org/10.1111/j.1365-2664.2011.02087.x"&gt;https://doi.org/10.1111/j.1365-2664.2011.02087.x&lt;/a&gt;
+&lt;br&gt;&lt;br&gt;
+Legendre, P., &amp;amp; Legendre, L. (1998). &lt;em&gt;Numerical Ecology&lt;/em&gt; (2nd English ed., Vol. 20). Elsevier.
+&lt;br&gt;&lt;br&gt;
+Manel, S., Williams, H. C., &amp;amp; Ormerod, S. J. (2001). Evaluating presence–absence models in ecology: The need to account for prevalence. &lt;em&gt;Journal of Applied Ecology, 38&lt;/em&gt;(5), 921–931.
+&lt;br&gt;&lt;br&gt;
+Margossian, Gelman, A., &amp;amp; C., C. (2023). For how many iterations should we run Markov chain Monte Carlo? &lt;em&gt;arXiv preprint arXiv:2311.02726&lt;/em&gt;. &lt;a href="https://doi.org/10.48550/arXiv.2311.02726"&gt;https://doi.org/10.48550/arXiv.2311.02726&lt;/a&gt;
+&lt;br&gt;&lt;br&gt;
+Mouillot, D., Graham, N. A. J., Villéger, S., Mason, N. W. H., &amp;amp; Bellwood, D. R. (2013). A functional approach reveals community responses to disturbances. &lt;em&gt;Trends in Ecology &amp;amp; Evolution, 28&lt;/em&gt;(3), 167–177.
+&lt;br&gt;&lt;br&gt;
+Ovaskainen, O., Tikhonov, G., Norberg, A., Guillaume Blanchet, F., Duan, L., Dunson, D., Roslin, T., &amp;amp; Abrego, N. (2017). How to make more out of community data? A conceptual framework and its implementation as models and software. &lt;em&gt;Ecology Letters, 20&lt;/em&gt;(5), 561–576. &lt;a href="https://doi.org/10.1111/ele.12757"&gt;https://doi.org/10.1111/ele.12757&lt;/a&gt;
+&lt;br&gt;&lt;br&gt;
+Palomares, M., &amp;amp; Pauly, D. S. (2022). World Wide Web electronic publication. Version (08/2021). Available online: &lt;a href="https://www.sealifebase.org/"&gt;www.sealifebase.org&lt;/a&gt; (accessed 4 September 2021).
+&lt;br&gt;&lt;br&gt;
+Romanuk, T. N., Hayward, A., &amp;amp; Hutchings, J. A. (2011). Trophic level scales positively with body size in fishes. &lt;em&gt;Global Ecology and Biogeography, 20&lt;/em&gt;(2), 231–240. &lt;a href="https://doi.org/10.1111/j.1466-8238.2010.00579.x"&gt;https://doi.org/10.1111/j.1466-8238.2010.00579.x&lt;/a&gt;
+&lt;br&gt;&lt;br&gt;
+Spedicato, M. T., Massutí, E., Mérigot, B., Tserpes, G., Jadaud, A., &amp;amp; Relini, G. (2019). The MEDITS trawl survey specifications in an ecosystem approach to fishery management. &lt;em&gt;Scientia Marina, 83&lt;/em&gt;(S1), 9–20. &lt;a href="https://doi.org/10.3989/SCIMAR.04915.11X"&gt;https://doi.org/10.3989/SCIMAR.04915.11X&lt;/a&gt;
+&lt;br&gt;&lt;br&gt;
+Thorson, J. T., &amp;amp; van der Bijl, W. (2023). phylosem: A fast and simple R package for phylogenetic inference and trait imputation using phylogenetic structural equation models. &lt;em&gt;Journal of Evolutionary Biology, 36&lt;/em&gt;(10), 1357–1364. &lt;a href="https://doi.org/10.1111/jeb.14234"&gt;https://doi.org/10.1111/jeb.14234&lt;/a&gt;
+&lt;br&gt;&lt;br&gt;
+Tikhonov, G., Opedal, Ø. H., Abrego, N., Lehikoinen, A., de Jonge, M. M. J., Oksanen, J., &amp;amp; Ovaskainen, O. (2020a). Joint species distribution modelling with the r-package Hmsc. &lt;em&gt;Methods in Ecology and Evolution, 11&lt;/em&gt;(3), 442–447. &lt;a href="https://doi.org/10.1111/2041-210X.13345"&gt;https://doi.org/10.1111/2041-210X.13345&lt;/a&gt;
+&lt;br&gt;&lt;br&gt;
+Tikhonov, G., Opedal, Ø. H., Abrego, N., Lehikoinen, A., de Jonge, M. M. J., Oksanen, J., &amp;amp; Ovaskainen, O. (2020b). Joint species distribution modelling with the r-package Hmsc. &lt;em&gt;Methods in Ecology and Evolution, 11&lt;/em&gt;(3), 442–447. &lt;a href="https://doi.org/10.1111/2041-210X.13345"&gt;https://doi.org/10.1111/2041-210X.13345&lt;/a&gt;
+&lt;br&gt;&lt;br&gt;
+Tjur, T. (2009). Coefficients of determination in logistic regression models - A new proposal: The coefficient of discrimination. &lt;em&gt;American Statistician, 63&lt;/em&gt;(4), 366–372. &lt;a href="https://doi.org/10.1198/TAST.2009.08210"&gt;https://doi.org/10.1198/TAST.2009.08210&lt;/a&gt;
+&lt;br&gt;&lt;br&gt;
+Vasquez, M., Allen, H., Manca, E., Castle, L., Lillis, H., Agnesi, S., Al Hamdani, Z., Annunziatellis, A., Askew, N., &amp;amp; Bekkby, T. (2021). &lt;em&gt;EUSeaMap 2021. A European broad-scale seabed habitat map&lt;/em&gt;.&lt;/p&gt;</t>
   </si>
 </sst>
 </file>
@@ -1111,14 +1036,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFAC5F67-39A2-465C-88B9-4321F2EB8BB8}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="143.54296875" customWidth="1"/>
-    <col min="3" max="3" width="85.26953125" customWidth="1"/>
+    <col min="1" max="1" width="18.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="143.5703125" customWidth="1"/>
+    <col min="3" max="3" width="85.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -1126,7 +1051,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="88.5" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1134,7 +1059,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="59" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -1142,7 +1067,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="44.25" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -1150,7 +1075,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="409.5" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>42</v>
       </c>
@@ -1158,7 +1083,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -1166,7 +1091,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="44.25" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1174,7 +1099,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1182,7 +1107,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="132.75" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>25</v>
       </c>
@@ -1190,7 +1115,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B10" s="1"/>
     </row>
   </sheetData>
@@ -1202,13 +1127,13 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A5808B4-DED8-4038-83E2-89CC5F8B5437}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="32.08984375" customWidth="1"/>
-    <col min="2" max="2" width="134.26953125" customWidth="1"/>
+    <col min="1" max="1" width="32.140625" customWidth="1"/>
+    <col min="2" max="2" width="134.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -1216,47 +1141,47 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>73</v>
       </c>
       <c r="B2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="162.25" x14ac:dyDescent="0.75">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="165" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>77</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="147.5" x14ac:dyDescent="0.75">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>79</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="206.5" x14ac:dyDescent="0.75">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>81</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="383.5" x14ac:dyDescent="0.75">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="390" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>75</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>76</v>
       </c>
@@ -1269,13 +1194,13 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{532B325C-EC70-401B-9B81-E90568F4AE5E}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.08984375" customWidth="1"/>
-    <col min="2" max="2" width="197.26953125" customWidth="1"/>
+    <col min="1" max="1" width="15.140625" customWidth="1"/>
+    <col min="2" max="2" width="197.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -1283,7 +1208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="28.75" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" ht="28.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>73</v>
       </c>
@@ -1291,39 +1216,39 @@
         <v>89</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="409.5" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:2" ht="285" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>77</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="132.75" x14ac:dyDescent="0.75">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>79</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="354" x14ac:dyDescent="0.75">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>81</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="409.5" x14ac:dyDescent="0.75">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>75</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>76</v>
       </c>
@@ -1336,13 +1261,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCDFC4F4-DA9B-4676-B4E9-27438403FC6D}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.1328125" customWidth="1"/>
-    <col min="2" max="2" width="110.40625" customWidth="1"/>
+    <col min="1" max="1" width="14.140625" customWidth="1"/>
+    <col min="2" max="2" width="110.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -1350,7 +1275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="409.5" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>44</v>
       </c>
@@ -1366,13 +1291,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98953C5C-C579-44AD-B9BC-A1CB08652AFC}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.86328125" customWidth="1"/>
-    <col min="2" max="2" width="92.86328125" customWidth="1"/>
+    <col min="1" max="1" width="26.85546875" customWidth="1"/>
+    <col min="2" max="2" width="92.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -1380,7 +1305,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1388,7 +1313,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -1396,7 +1321,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -1404,7 +1329,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="77.45" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:2" ht="77.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -1412,7 +1337,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -1420,12 +1345,12 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -1433,7 +1358,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -1449,13 +1374,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7534530D-A73A-4258-8656-ECA9512F2226}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.40625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="77.86328125" customWidth="1"/>
+    <col min="1" max="1" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="77.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -1463,7 +1388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="44.25" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -1471,7 +1396,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="73.75" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:2" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>46</v>
       </c>
@@ -1479,7 +1404,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="177" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>49</v>
       </c>
@@ -1487,7 +1412,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>66</v>
       </c>
@@ -1495,7 +1420,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>67</v>
       </c>
@@ -1503,7 +1428,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>68</v>
       </c>
@@ -1519,12 +1444,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24344193-A5DC-4C09-A7D0-962941565ADB}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="60.26953125" customWidth="1"/>
+    <col min="2" max="2" width="60.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -1532,7 +1457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -1540,7 +1465,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>28</v>
       </c>
@@ -1548,7 +1473,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>29</v>
       </c>
@@ -1556,7 +1481,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>30</v>
       </c>
@@ -1564,7 +1489,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>31</v>
       </c>
@@ -1572,7 +1497,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -1580,7 +1505,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>33</v>
       </c>
@@ -1597,12 +1522,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D71172A-305B-48CD-890B-1E71821EDF52}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="95.54296875" customWidth="1"/>
+    <col min="2" max="2" width="95.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -1610,7 +1535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="221.25" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" ht="225" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>56</v>
       </c>
@@ -1618,7 +1543,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="103.25" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>57</v>
       </c>
@@ -1626,7 +1551,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="103.25" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>58</v>
       </c>
@@ -1634,7 +1559,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="88.5" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>59</v>
       </c>
@@ -1642,7 +1567,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="103.25" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:2" ht="105" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>60</v>
       </c>
@@ -1658,13 +1583,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52622770-8B11-4F83-8FC4-BE5BFE84B716}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.54296875" customWidth="1"/>
+    <col min="1" max="1" width="25.5703125" customWidth="1"/>
     <col min="2" max="2" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -1672,7 +1597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>34</v>
       </c>
@@ -1688,12 +1613,12 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56BED128-4941-403A-8B14-BE1B70CB049C}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="149.54296875" customWidth="1"/>
+    <col min="2" max="2" width="149.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -1701,7 +1626,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="29.5" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>73</v>
       </c>
@@ -1709,7 +1634,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>77</v>
       </c>
@@ -1717,7 +1642,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="409.5" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>79</v>
       </c>
@@ -1725,7 +1650,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="132.75" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:2" ht="150" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>81</v>
       </c>
@@ -1733,7 +1658,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="409.5" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:2" ht="225" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>75</v>
       </c>
@@ -1741,7 +1666,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>76</v>
       </c>
@@ -1754,13 +1679,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19212195-0A71-4EBF-B930-11848C857DE8}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.6328125" customWidth="1"/>
-    <col min="2" max="2" width="149.6328125" customWidth="1"/>
+    <col min="1" max="1" width="17.5703125" customWidth="1"/>
+    <col min="2" max="2" width="149.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -1768,7 +1693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="58.75" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="2" spans="1:2" ht="58.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>73</v>
       </c>
@@ -1776,7 +1701,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="295" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:2" ht="300" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>77</v>
       </c>
@@ -1784,7 +1709,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="206.5" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:2" ht="210" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>79</v>
       </c>
@@ -1792,7 +1717,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="368.75" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:2" ht="375" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>81</v>
       </c>
@@ -1800,7 +1725,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="409.5" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:2" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>75</v>
       </c>
@@ -1808,7 +1733,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>76</v>
       </c>

</xml_diff>